<commit_message>
feat: add settings updater modal
</commit_message>
<xml_diff>
--- a/scripts/translations.xlsx
+++ b/scripts/translations.xlsx
@@ -1,131 +1,275 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tgim\grim-project\scripts\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{907EB1B9-755D-4AAB-8953-53C2D02834FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="42150" yWindow="0" windowWidth="12340" windowHeight="7730" xr2:uid="{345D26D2-1573-4113-A8BB-4B602D34706A}"/>
+    <workbookView xWindow="42150" yWindow="0" windowWidth="12340" windowHeight="7730"/>
   </bookViews>
   <sheets>
-    <sheet name="common" sheetId="1" r:id="rId1"/>
-    <sheet name="moa" sheetId="2" r:id="rId2"/>
+    <sheet sheetId="1" name="common" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="moa" state="visible" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="90">
   <si>
     <t>key</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>ko</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>en</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>jp</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>app_name</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GRIM</t>
+  </si>
+  <si>
+    <t>vault_name</t>
   </si>
   <si>
     <t>moa</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>GRIM</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>back</t>
+  </si>
+  <si>
+    <t>이전으로 돌아가기</t>
+  </si>
+  <si>
+    <t>settings.title</t>
+  </si>
+  <si>
+    <t>설정</t>
+  </si>
+  <si>
+    <t>Settings</t>
+  </si>
+  <si>
+    <t>設定</t>
+  </si>
+  <si>
+    <t>settings.close</t>
+  </si>
+  <si>
+    <t>설정 닫기</t>
+  </si>
+  <si>
+    <t>Close settings</t>
+  </si>
+  <si>
+    <t>設定を閉じる</t>
+  </si>
+  <si>
+    <t>settings.current_version</t>
+  </si>
+  <si>
+    <t>현재 버전</t>
+  </si>
+  <si>
+    <t>Current version</t>
+  </si>
+  <si>
+    <t>現在のバージョン</t>
+  </si>
+  <si>
+    <t>settings.check_for_updates</t>
+  </si>
+  <si>
+    <t>업데이트 확인</t>
+  </si>
+  <si>
+    <t>Check for updates</t>
+  </si>
+  <si>
+    <t>更新を確認</t>
+  </si>
+  <si>
+    <t>settings.checking_for_updates</t>
+  </si>
+  <si>
+    <t>업데이트 확인 중… {{progress}}%</t>
+  </si>
+  <si>
+    <t>Checking for updates… {{progress}}%</t>
+  </si>
+  <si>
+    <t>更新を確認中… {{progress}}%</t>
+  </si>
+  <si>
+    <t>settings.language</t>
+  </si>
+  <si>
+    <t>언어</t>
+  </si>
+  <si>
+    <t>Language</t>
+  </si>
+  <si>
+    <t>言語</t>
+  </si>
+  <si>
+    <t>settings.language_help</t>
+  </si>
+  <si>
+    <t>표시 언어를 선택합니다.</t>
+  </si>
+  <si>
+    <t>Choose the display language.</t>
+  </si>
+  <si>
+    <t>表示言語を選択します。</t>
+  </si>
+  <si>
+    <t>settings.done</t>
+  </si>
+  <si>
+    <t>완료</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>完了</t>
+  </si>
+  <si>
+    <t>settings.update_status.unsupported</t>
+  </si>
+  <si>
+    <t>업데이트 확인은 데스크톱 앱에서 사용할 수 있습니다.</t>
+  </si>
+  <si>
+    <t>Update checks are available in the desktop app.</t>
+  </si>
+  <si>
+    <t>更新確認はデスクトップアプリで利用できます。</t>
+  </si>
+  <si>
+    <t>settings.update_status.up_to_date</t>
+  </si>
+  <si>
+    <t>이미 최신 버전입니다.</t>
+  </si>
+  <si>
+    <t>You are already on the latest version.</t>
+  </si>
+  <si>
+    <t>すでに最新バージョンです。</t>
+  </si>
+  <si>
+    <t>settings.update_status.downloading</t>
+  </si>
+  <si>
+    <t>업데이트 다운로드 중…</t>
+  </si>
+  <si>
+    <t>Downloading update…</t>
+  </si>
+  <si>
+    <t>更新をダウンロード中…</t>
+  </si>
+  <si>
+    <t>settings.update_status.downloading_with_progress</t>
+  </si>
+  <si>
+    <t>업데이트 다운로드 중… {{progress}}%</t>
+  </si>
+  <si>
+    <t>Downloading update… {{progress}}%</t>
+  </si>
+  <si>
+    <t>更新をダウンロード中… {{progress}}%</t>
+  </si>
+  <si>
+    <t>settings.update_status.installing</t>
+  </si>
+  <si>
+    <t>업데이트 설치 중…</t>
+  </si>
+  <si>
+    <t>Installing update…</t>
+  </si>
+  <si>
+    <t>更新をインストール中…</t>
+  </si>
+  <si>
+    <t>settings.update_status.restarting</t>
+  </si>
+  <si>
+    <t>앱 재시작 중…</t>
+  </si>
+  <si>
+    <t>Restarting app…</t>
+  </si>
+  <si>
+    <t>アプリを再起動中…</t>
+  </si>
+  <si>
+    <t>settings.update_status.error</t>
+  </si>
+  <si>
+    <t>업데이트 확인에 실패했습니다.</t>
+  </si>
+  <si>
+    <t>Update failed.</t>
+  </si>
+  <si>
+    <t>更新に失敗しました。</t>
   </si>
   <si>
     <t>start_prompt</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>어떻게 시작하시겠어요?</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>How would you like to get started?</t>
+  </si>
+  <si>
+    <t>どのように始めますか？</t>
   </si>
   <si>
     <t>new_repository</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>새로운 레퍼런스 보관함 생성</t>
+  </si>
+  <si>
+    <t>Create a new reference folder</t>
+  </si>
+  <si>
+    <t>新しいリファレンスボールトを作成</t>
+  </si>
+  <si>
+    <t>new_repository_prompt</t>
+  </si>
+  <si>
+    <t>선택한 폴더 안에 새로운 {{vault_name}}를 생성합니다.</t>
+  </si>
+  <si>
+    <t>Create a new {{vault_name}} in the selected folder.</t>
+  </si>
+  <si>
+    <t>選択したフォルダーに新しい{{vault_name}}を作成します。</t>
   </si>
   <si>
     <t>import_repository</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>vault_name</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>new_repository_prompt</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>import_repository_prompt</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>레퍼런스 보관함 가져오기</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>새로운 레퍼런스 보관함 생성</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>선택한 폴더내에서 이미 존재하는 {{vault_name}}를 가져옵니다.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>선택한 폴더 안에 새로운 {{vault_name}}를 생성합니다.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>How would you like to get started?</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>どのように始めますか？</t>
-  </si>
-  <si>
-    <t>新しいリファレンスボールトを作成</t>
-  </si>
-  <si>
-    <t>選択したフォルダーに新しい{{vault_name}}を作成します。</t>
-  </si>
-  <si>
-    <t>Create a new {{vault_name}} in the selected folder.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Import reference folder</t>
   </si>
   <si>
     <r>
@@ -133,51 +277,55 @@
     </r>
     <r>
       <rPr>
+        <charset val="129"/>
+        <color theme="1"/>
+        <family val="3"/>
         <sz val="11"/>
-        <color theme="1"/>
         <rFont val="Noto Sans KR"/>
-        <family val="3"/>
-        <charset val="129"/>
       </rPr>
       <t>ー</t>
     </r>
     <r>
       <rPr>
+        <charset val="129"/>
+        <color theme="1"/>
+        <family val="3"/>
+        <scheme val="minor"/>
         <sz val="11"/>
-        <color theme="1"/>
         <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
       </rPr>
       <t>ルトをインポ</t>
     </r>
     <r>
       <rPr>
+        <charset val="129"/>
+        <color theme="1"/>
+        <family val="3"/>
         <sz val="11"/>
-        <color theme="1"/>
         <rFont val="Noto Sans KR"/>
-        <family val="3"/>
-        <charset val="129"/>
       </rPr>
       <t>ー</t>
     </r>
     <r>
       <rPr>
+        <charset val="129"/>
+        <color theme="1"/>
+        <family val="3"/>
+        <scheme val="minor"/>
         <sz val="11"/>
-        <color theme="1"/>
         <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
       </rPr>
       <t>ト</t>
     </r>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>import_repository_prompt</t>
+  </si>
+  <si>
+    <t>선택한 폴더내에서 이미 존재하는 {{vault_name}}를 가져옵니다.</t>
   </si>
   <si>
     <t>Import an existing {{vault_name}} from the selected folder.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -185,116 +333,77 @@
     </r>
     <r>
       <rPr>
+        <charset val="128"/>
+        <color theme="1"/>
+        <family val="2"/>
         <sz val="11"/>
-        <color theme="1"/>
         <rFont val="Yu Gothic"/>
-        <family val="2"/>
-        <charset val="128"/>
       </rPr>
       <t>択したフォルダーから既存の</t>
     </r>
     <r>
       <rPr>
+        <charset val="129"/>
+        <color theme="1"/>
+        <family val="2"/>
+        <scheme val="minor"/>
         <sz val="11"/>
-        <color theme="1"/>
         <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
       </rPr>
       <t>{{vault_name}}をインポ</t>
     </r>
     <r>
       <rPr>
+        <charset val="128"/>
+        <color theme="1"/>
+        <family val="2"/>
         <sz val="11"/>
-        <color theme="1"/>
         <rFont val="Yu Gothic"/>
-        <family val="2"/>
-        <charset val="128"/>
       </rPr>
       <t>ートします。</t>
     </r>
     <r>
       <rPr>
+        <charset val="129"/>
+        <color theme="1"/>
+        <family val="2"/>
+        <scheme val="minor"/>
         <sz val="11"/>
-        <color theme="1"/>
         <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
 </t>
     </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Create a new reference folder</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Import reference folder</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>back</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>이전으로 돌아가기</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
-      <charset val="129"/>
-      <scheme val="minor"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <sz val="8"/>
+      <charset val="129"/>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="11"/>
       <name val="맑은 고딕"/>
-      <family val="2"/>
-      <charset val="129"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <charset val="129"/>
+      <color theme="1"/>
+      <family val="3"/>
+      <scheme val="minor"/>
       <sz val="11"/>
-      <color theme="1"/>
       <name val="맑은 고딕"/>
-      <family val="3"/>
-      <charset val="129"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="맑은 고딕"/>
-      <family val="3"/>
-      <charset val="129"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Noto Sans KR"/>
-      <family val="3"/>
-      <charset val="129"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Yu Gothic"/>
-      <family val="2"/>
-      <charset val="128"/>
     </font>
   </fonts>
   <fills count="2">
@@ -315,15 +424,11 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -331,7 +436,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -662,9 +767,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B5E4D2A-23B7-4A5F-BC39-3B981A2919AF}">
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr defaultRowHeight="16.9" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.6" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="19.9375" customWidth="1"/>
     <col min="2" max="2" width="25.9375" customWidth="1"/>
@@ -672,7 +777,7 @@
     <col min="4" max="4" width="22.6875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.6">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -686,61 +791,270 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.6">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
         <v>11</v>
       </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.6">
-      <c r="A4" t="s">
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" t="s">
         <v>28</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D9" t="s">
         <v>29</v>
       </c>
     </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>50</v>
+      </c>
+      <c r="B15" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>58</v>
+      </c>
+      <c r="B17" t="s">
+        <v>59</v>
+      </c>
+      <c r="C17" t="s">
+        <v>60</v>
+      </c>
+      <c r="D17" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>62</v>
+      </c>
+      <c r="B18" t="s">
+        <v>63</v>
+      </c>
+      <c r="C18" t="s">
+        <v>64</v>
+      </c>
+      <c r="D18" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>66</v>
+      </c>
+      <c r="B19" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" t="s">
+        <v>68</v>
+      </c>
+      <c r="D19" t="s">
+        <v>69</v>
+      </c>
+    </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE50E907-B306-4A3B-929F-5C9BC904BB76}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
+  <sheetFormatPr defaultRowHeight="16.9" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.6" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="29.0625" style="1" customWidth="1"/>
     <col min="2" max="2" width="35.75" style="1" customWidth="1"/>
     <col min="3" max="3" width="22.0625" style="1" customWidth="1"/>
     <col min="4" max="4" width="20.25" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="9" style="1"/>
+    <col min="5" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.6">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -754,78 +1068,77 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="33.75" x14ac:dyDescent="0.6">
+    <row r="2" ht="33.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>7</v>
+        <v>70</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>8</v>
+        <v>71</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>18</v>
+        <v>72</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="33.75" x14ac:dyDescent="0.6">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" ht="33.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>9</v>
+        <v>74</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>26</v>
+        <v>76</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="50.65" x14ac:dyDescent="0.6">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="4" ht="50.65" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>12</v>
+        <v>78</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>17</v>
+        <v>79</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>22</v>
+        <v>80</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="36" x14ac:dyDescent="0.6">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>10</v>
+        <v>82</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>14</v>
+        <v>83</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>27</v>
+        <v>84</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="70.5" x14ac:dyDescent="0.6">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" ht="70.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>13</v>
+        <v>86</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>16</v>
+        <v>87</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>24</v>
+        <v>88</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>25</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(croquis): add custom window controls
</commit_message>
<xml_diff>
--- a/scripts/translations.xlsx
+++ b/scripts/translations.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1652" uniqueCount="1590">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1660" uniqueCount="1598">
   <si>
     <t>key</t>
   </si>
@@ -4781,6 +4781,30 @@
   </si>
   <si>
     <t>記録タグの更新に失敗しました。</t>
+  </si>
+  <si>
+    <t>common.minimize</t>
+  </si>
+  <si>
+    <t>Minimize</t>
+  </si>
+  <si>
+    <t>최소화</t>
+  </si>
+  <si>
+    <t>最小化</t>
+  </si>
+  <si>
+    <t>croquis.window_controls</t>
+  </si>
+  <si>
+    <t>Window controls</t>
+  </si>
+  <si>
+    <t>창 컨트롤</t>
+  </si>
+  <si>
+    <t>ウィンドウ操作</t>
   </si>
 </sst>
 </file>
@@ -5174,8 +5198,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D413"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac">
+  <dimension ref="A1:D415"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="48" customWidth="1"/>
@@ -10964,6 +10988,34 @@
         <v>1589</v>
       </c>
     </row>
+    <row r="414" ht="18" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A414" s="3" t="s">
+        <v>1590</v>
+      </c>
+      <c r="B414" s="3" t="s">
+        <v>1591</v>
+      </c>
+      <c r="C414" s="3" t="s">
+        <v>1592</v>
+      </c>
+      <c r="D414" s="3" t="s">
+        <v>1593</v>
+      </c>
+    </row>
+    <row r="415" ht="18" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A415" s="3" t="s">
+        <v>1594</v>
+      </c>
+      <c r="B415" s="3" t="s">
+        <v>1595</v>
+      </c>
+      <c r="C415" s="3" t="s">
+        <v>1596</v>
+      </c>
+      <c r="D415" s="3" t="s">
+        <v>1597</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
chore(i18n): add record export strings
</commit_message>
<xml_diff>
--- a/scripts/translations.xlsx
+++ b/scripts/translations.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1660" uniqueCount="1598">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1956" uniqueCount="1864">
   <si>
     <t>key</t>
   </si>
@@ -4805,6 +4805,804 @@
   </si>
   <si>
     <t>ウィンドウ操作</t>
+  </si>
+  <si>
+    <t>common.loading</t>
+  </si>
+  <si>
+    <t>Loading...</t>
+  </si>
+  <si>
+    <t>불러오는 중...</t>
+  </si>
+  <si>
+    <t>読み込み中...</t>
+  </si>
+  <si>
+    <t>common.browse</t>
+  </si>
+  <si>
+    <t>Browse</t>
+  </si>
+  <si>
+    <t>찾아보기</t>
+  </si>
+  <si>
+    <t>参照</t>
+  </si>
+  <si>
+    <t>record_export.title</t>
+  </si>
+  <si>
+    <t>Export Records</t>
+  </si>
+  <si>
+    <t>기록 내보내기</t>
+  </si>
+  <si>
+    <t>記録を書き出し</t>
+  </si>
+  <si>
+    <t>record_export.ratio.original</t>
+  </si>
+  <si>
+    <t>元の比率</t>
+  </si>
+  <si>
+    <t>record_export.ratio.custom</t>
+  </si>
+  <si>
+    <t>Custom</t>
+  </si>
+  <si>
+    <t>사용자 지정</t>
+  </si>
+  <si>
+    <t>カスタム</t>
+  </si>
+  <si>
+    <t>record_export.error.open_directory</t>
+  </si>
+  <si>
+    <t>Failed to open output folder picker.</t>
+  </si>
+  <si>
+    <t>출력 폴더 선택기를 열지 못했다.</t>
+  </si>
+  <si>
+    <t>出力フォルダー選択を開けませんでした。</t>
+  </si>
+  <si>
+    <t>record_export.error.export_failed</t>
+  </si>
+  <si>
+    <t>Failed to export selected records.</t>
+  </si>
+  <si>
+    <t>선택한 기록을 내보내지 못했다.</t>
+  </si>
+  <si>
+    <t>選択した記録を書き出せませんでした。</t>
+  </si>
+  <si>
+    <t>record_export.width</t>
+  </si>
+  <si>
+    <t>Width</t>
+  </si>
+  <si>
+    <t>너비</t>
+  </si>
+  <si>
+    <t>幅</t>
+  </si>
+  <si>
+    <t>record_export.height</t>
+  </si>
+  <si>
+    <t>Height</t>
+  </si>
+  <si>
+    <t>높이</t>
+  </si>
+  <si>
+    <t>高さ</t>
+  </si>
+  <si>
+    <t>record_export.use_ratio</t>
+  </si>
+  <si>
+    <t>Use ratio</t>
+  </si>
+  <si>
+    <t>비율 사용</t>
+  </si>
+  <si>
+    <t>比率を使用</t>
+  </si>
+  <si>
+    <t>record_export.ratio</t>
+  </si>
+  <si>
+    <t>Ratio</t>
+  </si>
+  <si>
+    <t>비율</t>
+  </si>
+  <si>
+    <t>比率</t>
+  </si>
+  <si>
+    <t>record_export.custom_ratio_width</t>
+  </si>
+  <si>
+    <t>Ratio W</t>
+  </si>
+  <si>
+    <t>비율 W</t>
+  </si>
+  <si>
+    <t>比率 W</t>
+  </si>
+  <si>
+    <t>record_export.custom_ratio_height</t>
+  </si>
+  <si>
+    <t>Ratio H</t>
+  </si>
+  <si>
+    <t>비율 H</t>
+  </si>
+  <si>
+    <t>比率 H</t>
+  </si>
+  <si>
+    <t>record_export.saved_to</t>
+  </si>
+  <si>
+    <t>Saved to {{path}}</t>
+  </si>
+  <si>
+    <t>{{path}}에 저장됨</t>
+  </si>
+  <si>
+    <t>{{path}} に保存しました</t>
+  </si>
+  <si>
+    <t>record_export.exporting</t>
+  </si>
+  <si>
+    <t>Exporting...</t>
+  </si>
+  <si>
+    <t>내보내는 중...</t>
+  </si>
+  <si>
+    <t>書き出し中...</t>
+  </si>
+  <si>
+    <t>record_export.export_png</t>
+  </si>
+  <si>
+    <t>Export PNG</t>
+  </si>
+  <si>
+    <t>PNG 내보내기</t>
+  </si>
+  <si>
+    <t>PNGを書き出し</t>
+  </si>
+  <si>
+    <t>record_export.selected_count</t>
+  </si>
+  <si>
+    <t>{{count}} selected</t>
+  </si>
+  <si>
+    <t>{{count}}개 선택됨</t>
+  </si>
+  <si>
+    <t>{{count}}件選択</t>
+  </si>
+  <si>
+    <t>record_export.exportable_count</t>
+  </si>
+  <si>
+    <t>{{count}} exportable</t>
+  </si>
+  <si>
+    <t>{{count}}개 내보내기 가능</t>
+  </si>
+  <si>
+    <t>{{count}}件書き出し可能</t>
+  </si>
+  <si>
+    <t>record_export.exported_count</t>
+  </si>
+  <si>
+    <t>{{count}} exported</t>
+  </si>
+  <si>
+    <t>{{count}}개 내보냄</t>
+  </si>
+  <si>
+    <t>{{count}}件書き出し済み</t>
+  </si>
+  <si>
+    <t>record_export.skipped_count</t>
+  </si>
+  <si>
+    <t>{{count}} skipped</t>
+  </si>
+  <si>
+    <t>{{count}}개 건너뜀</t>
+  </si>
+  <si>
+    <t>{{count}}件スキップ</t>
+  </si>
+  <si>
+    <t>record_export.no_exportable_records</t>
+  </si>
+  <si>
+    <t>Select records that have both source and result images.</t>
+  </si>
+  <si>
+    <t>원본과 결과 이미지가 모두 있는 기록을 선택해야 한다.</t>
+  </si>
+  <si>
+    <t>元画像と結果画像の両方がある記録を選択してください。</t>
+  </si>
+  <si>
+    <t>record_export.pair_layout</t>
+  </si>
+  <si>
+    <t>Pair layout</t>
+  </si>
+  <si>
+    <t>페어 레이아웃</t>
+  </si>
+  <si>
+    <t>ペアレイアウト</t>
+  </si>
+  <si>
+    <t>record_export.pair_layout_hint</t>
+  </si>
+  <si>
+    <t>Configure the source/result image boxes inside each record.</t>
+  </si>
+  <si>
+    <t>각 기록 안의 원본/결과 이미지 박스를 설정한다.</t>
+  </si>
+  <si>
+    <t>各記録内の元画像/結果画像ボックスを設定します。</t>
+  </si>
+  <si>
+    <t>record_export.source_image</t>
+  </si>
+  <si>
+    <t>Source image</t>
+  </si>
+  <si>
+    <t>원본 이미지</t>
+  </si>
+  <si>
+    <t>record_export.result_image</t>
+  </si>
+  <si>
+    <t>Result image</t>
+  </si>
+  <si>
+    <t>결과 이미지</t>
+  </si>
+  <si>
+    <t>結果画像</t>
+  </si>
+  <si>
+    <t>record_export.pair_spacing</t>
+  </si>
+  <si>
+    <t>Pair spacing</t>
+  </si>
+  <si>
+    <t>페어 간격</t>
+  </si>
+  <si>
+    <t>ペアの余白</t>
+  </si>
+  <si>
+    <t>record_export.gap</t>
+  </si>
+  <si>
+    <t>Gap</t>
+  </si>
+  <si>
+    <t>간격</t>
+  </si>
+  <si>
+    <t>間隔</t>
+  </si>
+  <si>
+    <t>record_export.padding</t>
+  </si>
+  <si>
+    <t>Padding</t>
+  </si>
+  <si>
+    <t>패딩</t>
+  </si>
+  <si>
+    <t>パディング</t>
+  </si>
+  <si>
+    <t>record_export.horizontal</t>
+  </si>
+  <si>
+    <t>Horizontal layout</t>
+  </si>
+  <si>
+    <t>가로 레이아웃</t>
+  </si>
+  <si>
+    <t>横並びレイアウト</t>
+  </si>
+  <si>
+    <t>record_export.grid_layout</t>
+  </si>
+  <si>
+    <t>Grid layout</t>
+  </si>
+  <si>
+    <t>그리드 레이아웃</t>
+  </si>
+  <si>
+    <t>グリッドレイアウト</t>
+  </si>
+  <si>
+    <t>record_export.grid_layout_hint</t>
+  </si>
+  <si>
+    <t>Arrange record blocks and select where the PNG will be saved.</t>
+  </si>
+  <si>
+    <t>기록 블록을 배치하고 PNG 저장 위치를 선택한다.</t>
+  </si>
+  <si>
+    <t>記録ブロックを配置し、PNGの保存先を選択します。</t>
+  </si>
+  <si>
+    <t>record_export.canvas_layout</t>
+  </si>
+  <si>
+    <t>Canvas layout</t>
+  </si>
+  <si>
+    <t>캔버스 레이아웃</t>
+  </si>
+  <si>
+    <t>キャンバスレイアウト</t>
+  </si>
+  <si>
+    <t>record_export.horizontal_gap</t>
+  </si>
+  <si>
+    <t>Horizontal gap</t>
+  </si>
+  <si>
+    <t>가로 간격</t>
+  </si>
+  <si>
+    <t>横の間隔</t>
+  </si>
+  <si>
+    <t>record_export.vertical_gap</t>
+  </si>
+  <si>
+    <t>Vertical gap</t>
+  </si>
+  <si>
+    <t>세로 간격</t>
+  </si>
+  <si>
+    <t>縦の間隔</t>
+  </si>
+  <si>
+    <t>record_export.outer_padding</t>
+  </si>
+  <si>
+    <t>Outer padding</t>
+  </si>
+  <si>
+    <t>전체 패딩</t>
+  </si>
+  <si>
+    <t>外側パディング</t>
+  </si>
+  <si>
+    <t>record_export.blocks_per_line</t>
+  </si>
+  <si>
+    <t>Blocks / line</t>
+  </si>
+  <si>
+    <t>한 줄당 블록</t>
+  </si>
+  <si>
+    <t>1行あたりのブロック</t>
+  </si>
+  <si>
+    <t>record_export.output</t>
+  </si>
+  <si>
+    <t>Output</t>
+  </si>
+  <si>
+    <t>출력</t>
+  </si>
+  <si>
+    <t>出力</t>
+  </si>
+  <si>
+    <t>record_export.output_folder</t>
+  </si>
+  <si>
+    <t>Output folder</t>
+  </si>
+  <si>
+    <t>출력 폴더</t>
+  </si>
+  <si>
+    <t>出力フォルダー</t>
+  </si>
+  <si>
+    <t>record_export.output_folder_placeholder</t>
+  </si>
+  <si>
+    <t>Choose a folder</t>
+  </si>
+  <si>
+    <t>record_export.file_name</t>
+  </si>
+  <si>
+    <t>File name</t>
+  </si>
+  <si>
+    <t>파일 이름</t>
+  </si>
+  <si>
+    <t>ファイル名</t>
+  </si>
+  <si>
+    <t>record_export.file_name_placeholder</t>
+  </si>
+  <si>
+    <t>grim-record-export-&lt;timestamp&gt;.png</t>
+  </si>
+  <si>
+    <t>record_export.preview</t>
+  </si>
+  <si>
+    <t>Preview</t>
+  </si>
+  <si>
+    <t>미리보기</t>
+  </si>
+  <si>
+    <t>プレビュー</t>
+  </si>
+  <si>
+    <t>record_export.canvas_size</t>
+  </si>
+  <si>
+    <t>Masonry, {{columns}} columns</t>
+  </si>
+  <si>
+    <t>Masonry, {{columns}}열</t>
+  </si>
+  <si>
+    <t>Masonry、{{columns}}列</t>
+  </si>
+  <si>
+    <t>record_export.default_file_name</t>
+  </si>
+  <si>
+    <t>record_export.ratio_mode</t>
+  </si>
+  <si>
+    <t>Ratio mode</t>
+  </si>
+  <si>
+    <t>비율 모드</t>
+  </si>
+  <si>
+    <t>比率モード</t>
+  </si>
+  <si>
+    <t>record_export.custom_w</t>
+  </si>
+  <si>
+    <t>Custom W</t>
+  </si>
+  <si>
+    <t>사용자 W</t>
+  </si>
+  <si>
+    <t>カスタム W</t>
+  </si>
+  <si>
+    <t>record_export.custom_h</t>
+  </si>
+  <si>
+    <t>Custom H</t>
+  </si>
+  <si>
+    <t>사용자 H</t>
+  </si>
+  <si>
+    <t>カスタム H</t>
+  </si>
+  <si>
+    <t>record_export.step_pair_title</t>
+  </si>
+  <si>
+    <t>Step 1 · Pair layout</t>
+  </si>
+  <si>
+    <t>Step 1 · 페어 레이아웃</t>
+  </si>
+  <si>
+    <t>Step 1 · ペアレイアウト</t>
+  </si>
+  <si>
+    <t>record_export.step_pair_hint</t>
+  </si>
+  <si>
+    <t>Configure how source and result images are placed in one record block.</t>
+  </si>
+  <si>
+    <t>원본과 결과 이미지가 하나의 기록 블록 안에 배치되는 방식을 설정한다.</t>
+  </si>
+  <si>
+    <t>元画像と結果画像を1つの記録ブロック内に配置する方法を設定します。</t>
+  </si>
+  <si>
+    <t>record_export.source_image_hint</t>
+  </si>
+  <si>
+    <t>Original image box settings</t>
+  </si>
+  <si>
+    <t>원본 이미지 박스 설정</t>
+  </si>
+  <si>
+    <t>元画像ボックス設定</t>
+  </si>
+  <si>
+    <t>record_export.result_image_hint</t>
+  </si>
+  <si>
+    <t>Captured result box settings</t>
+  </si>
+  <si>
+    <t>캡처된 결과 박스 설정</t>
+  </si>
+  <si>
+    <t>キャプチャ結果ボックス設定</t>
+  </si>
+  <si>
+    <t>record_export.pair_gap</t>
+  </si>
+  <si>
+    <t>Pair gap</t>
+  </si>
+  <si>
+    <t>ペア間隔</t>
+  </si>
+  <si>
+    <t>record_export.pair_padding</t>
+  </si>
+  <si>
+    <t>Pair padding</t>
+  </si>
+  <si>
+    <t>페어 패딩</t>
+  </si>
+  <si>
+    <t>ペアパディング</t>
+  </si>
+  <si>
+    <t>record_export.horizontal_alignment</t>
+  </si>
+  <si>
+    <t>Horizontal alignment</t>
+  </si>
+  <si>
+    <t>가로 정렬</t>
+  </si>
+  <si>
+    <t>横並び</t>
+  </si>
+  <si>
+    <t>record_export.pair_preview</t>
+  </si>
+  <si>
+    <t>Pair preview</t>
+  </si>
+  <si>
+    <t>페어 미리보기</t>
+  </si>
+  <si>
+    <t>ペアプレビュー</t>
+  </si>
+  <si>
+    <t>record_export.pair_preview_hint</t>
+  </si>
+  <si>
+    <t>One record block original and result inside padded export canvas</t>
+  </si>
+  <si>
+    <t>패딩이 적용된 export 캔버스 안의 기록 블록 원본과 결과</t>
+  </si>
+  <si>
+    <t>パディング付き書き出しキャンバス内の1記録ブロックの元画像と結果</t>
+  </si>
+  <si>
+    <t>record_export.source_label</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>record_export.result_label</t>
+  </si>
+  <si>
+    <t>record_export.no_preview</t>
+  </si>
+  <si>
+    <t>No preview available</t>
+  </si>
+  <si>
+    <t>미리보기가 없다</t>
+  </si>
+  <si>
+    <t>プレビューはありません</t>
+  </si>
+  <si>
+    <t>record_export.horizontal_short</t>
+  </si>
+  <si>
+    <t>Horizontal</t>
+  </si>
+  <si>
+    <t>record_export.vertical_short</t>
+  </si>
+  <si>
+    <t>Vertical</t>
+  </si>
+  <si>
+    <t>record_export.gap_value</t>
+  </si>
+  <si>
+    <t>Gap {{value}}px</t>
+  </si>
+  <si>
+    <t>record_export.padding_value</t>
+  </si>
+  <si>
+    <t>Padding {{value}}px</t>
+  </si>
+  <si>
+    <t>record_export.step_grid_title</t>
+  </si>
+  <si>
+    <t>Step 2 · Export grid</t>
+  </si>
+  <si>
+    <t>record_export.step_grid_hint</t>
+  </si>
+  <si>
+    <t>Choose output location and arrange all selected record blocks into one PNG.</t>
+  </si>
+  <si>
+    <t>출력 위치를 고르고 선택한 모든 기록 블록을 하나의 PNG로 배치한다.</t>
+  </si>
+  <si>
+    <t>出力先を選び、選択したすべての記録ブロックを1つのPNGに配置します。</t>
+  </si>
+  <si>
+    <t>record_export.final_export_grid</t>
+  </si>
+  <si>
+    <t>Final export grid</t>
+  </si>
+  <si>
+    <t>최종 export grid</t>
+  </si>
+  <si>
+    <t>最終書き出しグリッド</t>
+  </si>
+  <si>
+    <t>record_export.final_export_grid_hint</t>
+  </si>
+  <si>
+    <t>Masonry placement options for record blocks and output folder</t>
+  </si>
+  <si>
+    <t>기록 블록과 출력 폴더를 위한 masonry 배치 옵션</t>
+  </si>
+  <si>
+    <t>記録ブロックと出力フォルダーのMasonry配置オプション</t>
+  </si>
+  <si>
+    <t>record_export.columns</t>
+  </si>
+  <si>
+    <t>Columns</t>
+  </si>
+  <si>
+    <t>열</t>
+  </si>
+  <si>
+    <t>列</t>
+  </si>
+  <si>
+    <t>record_export.canvas_padding</t>
+  </si>
+  <si>
+    <t>Canvas padding</t>
+  </si>
+  <si>
+    <t>캔버스 패딩</t>
+  </si>
+  <si>
+    <t>キャンバスパディング</t>
+  </si>
+  <si>
+    <t>record_export.skip_incomplete</t>
+  </si>
+  <si>
+    <t>Skip records missing source or result image</t>
+  </si>
+  <si>
+    <t>원본 또는 결과 이미지가 없는 기록 건너뛰기</t>
+  </si>
+  <si>
+    <t>元画像または結果画像がない記録をスキップ</t>
+  </si>
+  <si>
+    <t>record_export.export_summary</t>
+  </si>
+  <si>
+    <t>Export summary</t>
+  </si>
+  <si>
+    <t>record_export.export_summary_hint</t>
+  </si>
+  <si>
+    <t>Only complete records are included in the PNG merge</t>
+  </si>
+  <si>
+    <t>완성된 기록만 PNG 병합에 포함된다.</t>
+  </si>
+  <si>
+    <t>完全な記録のみPNG結合に含まれます。</t>
+  </si>
+  <si>
+    <t>record_export.merged_png_preview</t>
+  </si>
+  <si>
+    <t>Merged PNG preview</t>
+  </si>
+  <si>
+    <t>record_export.merged_png_preview_hint</t>
+  </si>
+  <si>
+    <t>Masonry columns place each record block in the shortest column</t>
+  </si>
+  <si>
+    <t>Masonry 열은 각 기록 블록을 가장 짧은 열에 배치한다.</t>
+  </si>
+  <si>
+    <t>Masonry列は各記録ブロックを最も短い列に配置します。</t>
   </si>
 </sst>
 </file>
@@ -4824,7 +5622,7 @@
       <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4835,6 +5633,9 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF2F3437"/>
       </patternFill>
+    </fill>
+    <fill>
+      <patternFill/>
     </fill>
   </fills>
   <borders count="1">
@@ -4857,7 +5658,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5198,9 +5999,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac">
-  <dimension ref="A1:D415"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:D489"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="48" customWidth="1"/>
     <col min="2" max="4" width="72" customWidth="1"/>
@@ -11016,8 +11820,1044 @@
         <v>1597</v>
       </c>
     </row>
+    <row r="416" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A416" t="s">
+        <v>1598</v>
+      </c>
+      <c r="B416" t="s">
+        <v>1599</v>
+      </c>
+      <c r="C416" t="s">
+        <v>1600</v>
+      </c>
+      <c r="D416" t="s">
+        <v>1601</v>
+      </c>
+    </row>
+    <row r="417" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A417" t="s">
+        <v>1602</v>
+      </c>
+      <c r="B417" t="s">
+        <v>1603</v>
+      </c>
+      <c r="C417" t="s">
+        <v>1604</v>
+      </c>
+      <c r="D417" t="s">
+        <v>1605</v>
+      </c>
+    </row>
+    <row r="418" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A418" t="s">
+        <v>1606</v>
+      </c>
+      <c r="B418" t="s">
+        <v>1607</v>
+      </c>
+      <c r="C418" t="s">
+        <v>1608</v>
+      </c>
+      <c r="D418" t="s">
+        <v>1609</v>
+      </c>
+    </row>
+    <row r="419" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A419" t="s">
+        <v>1610</v>
+      </c>
+      <c r="B419" t="s">
+        <v>1152</v>
+      </c>
+      <c r="C419" t="s">
+        <v>1153</v>
+      </c>
+      <c r="D419" t="s">
+        <v>1611</v>
+      </c>
+    </row>
+    <row r="420" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A420" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B420" t="s">
+        <v>1613</v>
+      </c>
+      <c r="C420" t="s">
+        <v>1614</v>
+      </c>
+      <c r="D420" t="s">
+        <v>1615</v>
+      </c>
+    </row>
+    <row r="421" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A421" t="s">
+        <v>1616</v>
+      </c>
+      <c r="B421" t="s">
+        <v>1617</v>
+      </c>
+      <c r="C421" t="s">
+        <v>1618</v>
+      </c>
+      <c r="D421" t="s">
+        <v>1619</v>
+      </c>
+    </row>
+    <row r="422" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A422" t="s">
+        <v>1620</v>
+      </c>
+      <c r="B422" t="s">
+        <v>1621</v>
+      </c>
+      <c r="C422" t="s">
+        <v>1622</v>
+      </c>
+      <c r="D422" t="s">
+        <v>1623</v>
+      </c>
+    </row>
+    <row r="423" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A423" t="s">
+        <v>1624</v>
+      </c>
+      <c r="B423" t="s">
+        <v>1625</v>
+      </c>
+      <c r="C423" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D423" t="s">
+        <v>1627</v>
+      </c>
+    </row>
+    <row r="424" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A424" t="s">
+        <v>1628</v>
+      </c>
+      <c r="B424" t="s">
+        <v>1629</v>
+      </c>
+      <c r="C424" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D424" t="s">
+        <v>1631</v>
+      </c>
+    </row>
+    <row r="425" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A425" t="s">
+        <v>1632</v>
+      </c>
+      <c r="B425" t="s">
+        <v>1633</v>
+      </c>
+      <c r="C425" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D425" t="s">
+        <v>1635</v>
+      </c>
+    </row>
+    <row r="426" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A426" t="s">
+        <v>1636</v>
+      </c>
+      <c r="B426" t="s">
+        <v>1637</v>
+      </c>
+      <c r="C426" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D426" t="s">
+        <v>1639</v>
+      </c>
+    </row>
+    <row r="427" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A427" t="s">
+        <v>1640</v>
+      </c>
+      <c r="B427" t="s">
+        <v>1641</v>
+      </c>
+      <c r="C427" t="s">
+        <v>1642</v>
+      </c>
+      <c r="D427" t="s">
+        <v>1643</v>
+      </c>
+    </row>
+    <row r="428" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A428" t="s">
+        <v>1644</v>
+      </c>
+      <c r="B428" t="s">
+        <v>1645</v>
+      </c>
+      <c r="C428" t="s">
+        <v>1646</v>
+      </c>
+      <c r="D428" t="s">
+        <v>1647</v>
+      </c>
+    </row>
+    <row r="429" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A429" t="s">
+        <v>1648</v>
+      </c>
+      <c r="B429" t="s">
+        <v>1649</v>
+      </c>
+      <c r="C429" t="s">
+        <v>1650</v>
+      </c>
+      <c r="D429" t="s">
+        <v>1651</v>
+      </c>
+    </row>
+    <row r="430" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A430" t="s">
+        <v>1652</v>
+      </c>
+      <c r="B430" t="s">
+        <v>1653</v>
+      </c>
+      <c r="C430" t="s">
+        <v>1654</v>
+      </c>
+      <c r="D430" t="s">
+        <v>1655</v>
+      </c>
+    </row>
+    <row r="431" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A431" t="s">
+        <v>1656</v>
+      </c>
+      <c r="B431" t="s">
+        <v>1657</v>
+      </c>
+      <c r="C431" t="s">
+        <v>1658</v>
+      </c>
+      <c r="D431" t="s">
+        <v>1659</v>
+      </c>
+    </row>
+    <row r="432" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A432" t="s">
+        <v>1660</v>
+      </c>
+      <c r="B432" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C432" t="s">
+        <v>1662</v>
+      </c>
+      <c r="D432" t="s">
+        <v>1663</v>
+      </c>
+    </row>
+    <row r="433" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A433" t="s">
+        <v>1664</v>
+      </c>
+      <c r="B433" t="s">
+        <v>1665</v>
+      </c>
+      <c r="C433" t="s">
+        <v>1666</v>
+      </c>
+      <c r="D433" t="s">
+        <v>1667</v>
+      </c>
+    </row>
+    <row r="434" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A434" t="s">
+        <v>1668</v>
+      </c>
+      <c r="B434" t="s">
+        <v>1669</v>
+      </c>
+      <c r="C434" t="s">
+        <v>1670</v>
+      </c>
+      <c r="D434" t="s">
+        <v>1671</v>
+      </c>
+    </row>
+    <row r="435" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A435" t="s">
+        <v>1672</v>
+      </c>
+      <c r="B435" t="s">
+        <v>1673</v>
+      </c>
+      <c r="C435" t="s">
+        <v>1674</v>
+      </c>
+      <c r="D435" t="s">
+        <v>1675</v>
+      </c>
+    </row>
+    <row r="436" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A436" t="s">
+        <v>1676</v>
+      </c>
+      <c r="B436" t="s">
+        <v>1677</v>
+      </c>
+      <c r="C436" t="s">
+        <v>1678</v>
+      </c>
+      <c r="D436" t="s">
+        <v>1679</v>
+      </c>
+    </row>
+    <row r="437" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A437" t="s">
+        <v>1680</v>
+      </c>
+      <c r="B437" t="s">
+        <v>1681</v>
+      </c>
+      <c r="C437" t="s">
+        <v>1682</v>
+      </c>
+      <c r="D437" t="s">
+        <v>1683</v>
+      </c>
+    </row>
+    <row r="438" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A438" t="s">
+        <v>1684</v>
+      </c>
+      <c r="B438" t="s">
+        <v>1685</v>
+      </c>
+      <c r="C438" t="s">
+        <v>1686</v>
+      </c>
+      <c r="D438" t="s">
+        <v>1687</v>
+      </c>
+    </row>
+    <row r="439" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A439" t="s">
+        <v>1688</v>
+      </c>
+      <c r="B439" t="s">
+        <v>1689</v>
+      </c>
+      <c r="C439" t="s">
+        <v>1690</v>
+      </c>
+      <c r="D439" t="s">
+        <v>1154</v>
+      </c>
+    </row>
+    <row r="440" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A440" t="s">
+        <v>1691</v>
+      </c>
+      <c r="B440" t="s">
+        <v>1692</v>
+      </c>
+      <c r="C440" t="s">
+        <v>1693</v>
+      </c>
+      <c r="D440" t="s">
+        <v>1694</v>
+      </c>
+    </row>
+    <row r="441" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A441" t="s">
+        <v>1695</v>
+      </c>
+      <c r="B441" t="s">
+        <v>1696</v>
+      </c>
+      <c r="C441" t="s">
+        <v>1697</v>
+      </c>
+      <c r="D441" t="s">
+        <v>1698</v>
+      </c>
+    </row>
+    <row r="442" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A442" t="s">
+        <v>1699</v>
+      </c>
+      <c r="B442" t="s">
+        <v>1700</v>
+      </c>
+      <c r="C442" t="s">
+        <v>1701</v>
+      </c>
+      <c r="D442" t="s">
+        <v>1702</v>
+      </c>
+    </row>
+    <row r="443" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A443" t="s">
+        <v>1703</v>
+      </c>
+      <c r="B443" t="s">
+        <v>1704</v>
+      </c>
+      <c r="C443" t="s">
+        <v>1705</v>
+      </c>
+      <c r="D443" t="s">
+        <v>1706</v>
+      </c>
+    </row>
+    <row r="444" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A444" t="s">
+        <v>1707</v>
+      </c>
+      <c r="B444" t="s">
+        <v>1708</v>
+      </c>
+      <c r="C444" t="s">
+        <v>1709</v>
+      </c>
+      <c r="D444" t="s">
+        <v>1710</v>
+      </c>
+    </row>
+    <row r="445" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A445" t="s">
+        <v>1711</v>
+      </c>
+      <c r="B445" t="s">
+        <v>1712</v>
+      </c>
+      <c r="C445" t="s">
+        <v>1713</v>
+      </c>
+      <c r="D445" t="s">
+        <v>1714</v>
+      </c>
+    </row>
+    <row r="446" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A446" t="s">
+        <v>1715</v>
+      </c>
+      <c r="B446" t="s">
+        <v>1716</v>
+      </c>
+      <c r="C446" t="s">
+        <v>1717</v>
+      </c>
+      <c r="D446" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="447" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A447" t="s">
+        <v>1719</v>
+      </c>
+      <c r="B447" t="s">
+        <v>1720</v>
+      </c>
+      <c r="C447" t="s">
+        <v>1721</v>
+      </c>
+      <c r="D447" t="s">
+        <v>1722</v>
+      </c>
+    </row>
+    <row r="448" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A448" t="s">
+        <v>1723</v>
+      </c>
+      <c r="B448" t="s">
+        <v>1724</v>
+      </c>
+      <c r="C448" t="s">
+        <v>1725</v>
+      </c>
+      <c r="D448" t="s">
+        <v>1726</v>
+      </c>
+    </row>
+    <row r="449" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A449" t="s">
+        <v>1727</v>
+      </c>
+      <c r="B449" t="s">
+        <v>1728</v>
+      </c>
+      <c r="C449" t="s">
+        <v>1729</v>
+      </c>
+      <c r="D449" t="s">
+        <v>1730</v>
+      </c>
+    </row>
+    <row r="450" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A450" t="s">
+        <v>1731</v>
+      </c>
+      <c r="B450" t="s">
+        <v>1732</v>
+      </c>
+      <c r="C450" t="s">
+        <v>1733</v>
+      </c>
+      <c r="D450" t="s">
+        <v>1734</v>
+      </c>
+    </row>
+    <row r="451" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A451" t="s">
+        <v>1735</v>
+      </c>
+      <c r="B451" t="s">
+        <v>1736</v>
+      </c>
+      <c r="C451" t="s">
+        <v>1737</v>
+      </c>
+      <c r="D451" t="s">
+        <v>1738</v>
+      </c>
+    </row>
+    <row r="452" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A452" t="s">
+        <v>1739</v>
+      </c>
+      <c r="B452" t="s">
+        <v>1740</v>
+      </c>
+      <c r="C452" t="s">
+        <v>1741</v>
+      </c>
+      <c r="D452" t="s">
+        <v>1742</v>
+      </c>
+    </row>
+    <row r="453" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A453" t="s">
+        <v>1743</v>
+      </c>
+      <c r="B453" t="s">
+        <v>1744</v>
+      </c>
+      <c r="C453" t="s">
+        <v>1745</v>
+      </c>
+      <c r="D453" t="s">
+        <v>1746</v>
+      </c>
+    </row>
+    <row r="454" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A454" t="s">
+        <v>1747</v>
+      </c>
+      <c r="B454" t="s">
+        <v>1748</v>
+      </c>
+      <c r="C454" t="s">
+        <v>828</v>
+      </c>
+      <c r="D454" t="s">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="455" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A455" t="s">
+        <v>1749</v>
+      </c>
+      <c r="B455" t="s">
+        <v>1750</v>
+      </c>
+      <c r="C455" t="s">
+        <v>1751</v>
+      </c>
+      <c r="D455" t="s">
+        <v>1752</v>
+      </c>
+    </row>
+    <row r="456" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A456" t="s">
+        <v>1753</v>
+      </c>
+      <c r="B456" t="s">
+        <v>1754</v>
+      </c>
+      <c r="C456" t="s">
+        <v>1754</v>
+      </c>
+      <c r="D456" t="s">
+        <v>1754</v>
+      </c>
+    </row>
+    <row r="457" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A457" t="s">
+        <v>1755</v>
+      </c>
+      <c r="B457" t="s">
+        <v>1756</v>
+      </c>
+      <c r="C457" t="s">
+        <v>1757</v>
+      </c>
+      <c r="D457" t="s">
+        <v>1758</v>
+      </c>
+    </row>
+    <row r="458" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A458" t="s">
+        <v>1759</v>
+      </c>
+      <c r="B458" t="s">
+        <v>1760</v>
+      </c>
+      <c r="C458" t="s">
+        <v>1761</v>
+      </c>
+      <c r="D458" t="s">
+        <v>1762</v>
+      </c>
+    </row>
+    <row r="459" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A459" t="s">
+        <v>1763</v>
+      </c>
+      <c r="B459" t="s">
+        <v>1754</v>
+      </c>
+      <c r="C459" t="s">
+        <v>1754</v>
+      </c>
+      <c r="D459" t="s">
+        <v>1754</v>
+      </c>
+    </row>
+    <row r="460" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A460" t="s">
+        <v>1764</v>
+      </c>
+      <c r="B460" t="s">
+        <v>1765</v>
+      </c>
+      <c r="C460" t="s">
+        <v>1766</v>
+      </c>
+      <c r="D460" t="s">
+        <v>1767</v>
+      </c>
+    </row>
+    <row r="461" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A461" t="s">
+        <v>1768</v>
+      </c>
+      <c r="B461" t="s">
+        <v>1769</v>
+      </c>
+      <c r="C461" t="s">
+        <v>1770</v>
+      </c>
+      <c r="D461" t="s">
+        <v>1771</v>
+      </c>
+    </row>
+    <row r="462" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A462" t="s">
+        <v>1772</v>
+      </c>
+      <c r="B462" t="s">
+        <v>1773</v>
+      </c>
+      <c r="C462" t="s">
+        <v>1774</v>
+      </c>
+      <c r="D462" t="s">
+        <v>1775</v>
+      </c>
+    </row>
+    <row r="463" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A463" t="s">
+        <v>1776</v>
+      </c>
+      <c r="B463" t="s">
+        <v>1777</v>
+      </c>
+      <c r="C463" t="s">
+        <v>1778</v>
+      </c>
+      <c r="D463" t="s">
+        <v>1779</v>
+      </c>
+    </row>
+    <row r="464" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A464" t="s">
+        <v>1780</v>
+      </c>
+      <c r="B464" t="s">
+        <v>1781</v>
+      </c>
+      <c r="C464" t="s">
+        <v>1782</v>
+      </c>
+      <c r="D464" t="s">
+        <v>1783</v>
+      </c>
+    </row>
+    <row r="465" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A465" t="s">
+        <v>1784</v>
+      </c>
+      <c r="B465" t="s">
+        <v>1785</v>
+      </c>
+      <c r="C465" t="s">
+        <v>1786</v>
+      </c>
+      <c r="D465" t="s">
+        <v>1787</v>
+      </c>
+    </row>
+    <row r="466" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A466" t="s">
+        <v>1788</v>
+      </c>
+      <c r="B466" t="s">
+        <v>1789</v>
+      </c>
+      <c r="C466" t="s">
+        <v>1790</v>
+      </c>
+      <c r="D466" t="s">
+        <v>1791</v>
+      </c>
+    </row>
+    <row r="467" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A467" t="s">
+        <v>1792</v>
+      </c>
+      <c r="B467" t="s">
+        <v>1793</v>
+      </c>
+      <c r="C467" t="s">
+        <v>1697</v>
+      </c>
+      <c r="D467" t="s">
+        <v>1794</v>
+      </c>
+    </row>
+    <row r="468" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A468" t="s">
+        <v>1795</v>
+      </c>
+      <c r="B468" t="s">
+        <v>1796</v>
+      </c>
+      <c r="C468" t="s">
+        <v>1797</v>
+      </c>
+      <c r="D468" t="s">
+        <v>1798</v>
+      </c>
+    </row>
+    <row r="469" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A469" t="s">
+        <v>1799</v>
+      </c>
+      <c r="B469" t="s">
+        <v>1800</v>
+      </c>
+      <c r="C469" t="s">
+        <v>1801</v>
+      </c>
+      <c r="D469" t="s">
+        <v>1802</v>
+      </c>
+    </row>
+    <row r="470" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A470" t="s">
+        <v>1803</v>
+      </c>
+      <c r="B470" t="s">
+        <v>1804</v>
+      </c>
+      <c r="C470" t="s">
+        <v>1805</v>
+      </c>
+      <c r="D470" t="s">
+        <v>1806</v>
+      </c>
+    </row>
+    <row r="471" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A471" t="s">
+        <v>1807</v>
+      </c>
+      <c r="B471" t="s">
+        <v>1808</v>
+      </c>
+      <c r="C471" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D471" t="s">
+        <v>1810</v>
+      </c>
+    </row>
+    <row r="472" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A472" t="s">
+        <v>1811</v>
+      </c>
+      <c r="B472" t="s">
+        <v>1812</v>
+      </c>
+      <c r="C472" t="s">
+        <v>1812</v>
+      </c>
+      <c r="D472" t="s">
+        <v>1812</v>
+      </c>
+    </row>
+    <row r="473" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A473" t="s">
+        <v>1813</v>
+      </c>
+      <c r="B473" t="s">
+        <v>1156</v>
+      </c>
+      <c r="C473" t="s">
+        <v>1156</v>
+      </c>
+      <c r="D473" t="s">
+        <v>1156</v>
+      </c>
+    </row>
+    <row r="474" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A474" t="s">
+        <v>1814</v>
+      </c>
+      <c r="B474" t="s">
+        <v>1815</v>
+      </c>
+      <c r="C474" t="s">
+        <v>1816</v>
+      </c>
+      <c r="D474" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="475" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A475" t="s">
+        <v>1818</v>
+      </c>
+      <c r="B475" t="s">
+        <v>1819</v>
+      </c>
+      <c r="C475" t="s">
+        <v>1819</v>
+      </c>
+      <c r="D475" t="s">
+        <v>1819</v>
+      </c>
+    </row>
+    <row r="476" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A476" t="s">
+        <v>1820</v>
+      </c>
+      <c r="B476" t="s">
+        <v>1821</v>
+      </c>
+      <c r="C476" t="s">
+        <v>1821</v>
+      </c>
+      <c r="D476" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="477" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A477" t="s">
+        <v>1822</v>
+      </c>
+      <c r="B477" t="s">
+        <v>1823</v>
+      </c>
+      <c r="C477" t="s">
+        <v>1823</v>
+      </c>
+      <c r="D477" t="s">
+        <v>1823</v>
+      </c>
+    </row>
+    <row r="478" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A478" t="s">
+        <v>1824</v>
+      </c>
+      <c r="B478" t="s">
+        <v>1825</v>
+      </c>
+      <c r="C478" t="s">
+        <v>1825</v>
+      </c>
+      <c r="D478" t="s">
+        <v>1825</v>
+      </c>
+    </row>
+    <row r="479" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A479" t="s">
+        <v>1826</v>
+      </c>
+      <c r="B479" t="s">
+        <v>1827</v>
+      </c>
+      <c r="C479" t="s">
+        <v>1827</v>
+      </c>
+      <c r="D479" t="s">
+        <v>1827</v>
+      </c>
+    </row>
+    <row r="480" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A480" t="s">
+        <v>1828</v>
+      </c>
+      <c r="B480" t="s">
+        <v>1829</v>
+      </c>
+      <c r="C480" t="s">
+        <v>1830</v>
+      </c>
+      <c r="D480" t="s">
+        <v>1831</v>
+      </c>
+    </row>
+    <row r="481" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A481" t="s">
+        <v>1832</v>
+      </c>
+      <c r="B481" t="s">
+        <v>1833</v>
+      </c>
+      <c r="C481" t="s">
+        <v>1834</v>
+      </c>
+      <c r="D481" t="s">
+        <v>1835</v>
+      </c>
+    </row>
+    <row r="482" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A482" t="s">
+        <v>1836</v>
+      </c>
+      <c r="B482" t="s">
+        <v>1837</v>
+      </c>
+      <c r="C482" t="s">
+        <v>1838</v>
+      </c>
+      <c r="D482" t="s">
+        <v>1839</v>
+      </c>
+    </row>
+    <row r="483" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A483" t="s">
+        <v>1840</v>
+      </c>
+      <c r="B483" t="s">
+        <v>1841</v>
+      </c>
+      <c r="C483" t="s">
+        <v>1842</v>
+      </c>
+      <c r="D483" t="s">
+        <v>1843</v>
+      </c>
+    </row>
+    <row r="484" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A484" t="s">
+        <v>1844</v>
+      </c>
+      <c r="B484" t="s">
+        <v>1845</v>
+      </c>
+      <c r="C484" t="s">
+        <v>1846</v>
+      </c>
+      <c r="D484" t="s">
+        <v>1847</v>
+      </c>
+    </row>
+    <row r="485" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A485" t="s">
+        <v>1848</v>
+      </c>
+      <c r="B485" t="s">
+        <v>1849</v>
+      </c>
+      <c r="C485" t="s">
+        <v>1850</v>
+      </c>
+      <c r="D485" t="s">
+        <v>1851</v>
+      </c>
+    </row>
+    <row r="486" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A486" t="s">
+        <v>1852</v>
+      </c>
+      <c r="B486" t="s">
+        <v>1853</v>
+      </c>
+      <c r="C486" t="s">
+        <v>1853</v>
+      </c>
+      <c r="D486" t="s">
+        <v>1853</v>
+      </c>
+    </row>
+    <row r="487" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A487" t="s">
+        <v>1854</v>
+      </c>
+      <c r="B487" t="s">
+        <v>1855</v>
+      </c>
+      <c r="C487" t="s">
+        <v>1856</v>
+      </c>
+      <c r="D487" t="s">
+        <v>1857</v>
+      </c>
+    </row>
+    <row r="488" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A488" t="s">
+        <v>1858</v>
+      </c>
+      <c r="B488" t="s">
+        <v>1859</v>
+      </c>
+      <c r="C488" t="s">
+        <v>1859</v>
+      </c>
+      <c r="D488" t="s">
+        <v>1859</v>
+      </c>
+    </row>
+    <row r="489" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A489" t="s">
+        <v>1860</v>
+      </c>
+      <c r="B489" t="s">
+        <v>1861</v>
+      </c>
+      <c r="C489" t="s">
+        <v>1862</v>
+      </c>
+      <c r="D489" t="s">
+        <v>1863</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>